<commit_message>
Completed Writing the project Specifications
A list for what is needed for each entity in the project, and can be used later for planning time allocation and creation.
</commit_message>
<xml_diff>
--- a/UserStoriesLatterHalf.xlsx
+++ b/UserStoriesLatterHalf.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luke\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jdthr\Downloads\Software-Engineering-Project-G1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4892E7B6-41DB-4CBD-A7A9-88B4F8DE2BB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43168BCB-0D22-4924-815E-1339CC675F82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1071,7 +1071,7 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B76" s="1" t="s">
         <v>45</v>
@@ -1098,7 +1098,7 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B80" s="1" t="s">
         <v>45</v>
@@ -1123,7 +1123,7 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B84" s="1" t="s">
         <v>45</v>

</xml_diff>